<commit_message>
feat: add comprehensive Playwright test suite, page objects, and test data for CRM validation
</commit_message>
<xml_diff>
--- a/testdata/lead/bulk_upload/admin_contact.xlsx
+++ b/testdata/lead/bulk_upload/admin_contact.xlsx
@@ -412,57 +412,57 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Deepesh Pandey</v>
+        <v>Anwesha Varrier</v>
       </c>
       <c r="B2" t="str">
-        <v>deepesh.pandey978@gmail.com</v>
+        <v>anwesha.varrier895@gmail.com</v>
       </c>
       <c r="C2">
-        <v>6333236108</v>
+        <v>7053029221</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Rita Pillai</v>
+        <v>Brahmdev Joshi</v>
       </c>
       <c r="B3" t="str">
-        <v>rita.pillai647@gmail.com</v>
+        <v>brahmdev.joshi380@gmail.com</v>
       </c>
       <c r="C3">
-        <v>9934057888</v>
+        <v>8877180993</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Mayoor Tandon</v>
+        <v>Akshaj Saini</v>
       </c>
       <c r="B4" t="str">
-        <v>mayoor.tandon744@gmail.com</v>
+        <v>akshaj.saini934@gmail.com</v>
       </c>
       <c r="C4">
-        <v>9668968303</v>
+        <v>6393109115</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Daiwik Varma</v>
+        <v>Rageshwari Bhattacharya</v>
       </c>
       <c r="B5" t="str">
-        <v>daiwik.varma686@gmail.com</v>
+        <v>rageshwari.bhattacharya100@gmail.com</v>
       </c>
       <c r="C5">
-        <v>9612568214</v>
+        <v>9669182759</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Ranjeet Bhattathiri</v>
+        <v>Siddarth Jain</v>
       </c>
       <c r="B6" t="str">
-        <v>ranjeet.bhattathiri575@gmail.com</v>
+        <v>siddarth.jain176@gmail.com</v>
       </c>
       <c r="C6">
-        <v>8772147681</v>
+        <v>9812365279</v>
       </c>
     </row>
   </sheetData>

</xml_diff>